<commit_message>
feat: implement aircraft metadata header, redesign layout flow and clean docs
</commit_message>
<xml_diff>
--- a/docs/Parâmetros de Aeronaves e Manutenção.xlsx
+++ b/docs/Parâmetros de Aeronaves e Manutenção.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bruno/Documents/Gemini/10_PROJETOS/VADER/docs/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\brgar\Projetos\VADER\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B5100CB-C3FC-E84E-8C6B-95A90906D5FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3520DD0E-5AF1-430C-91DC-B4E99960E03D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17220" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="16800" yWindow="0" windowWidth="24450" windowHeight="15345" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Parâmetros de Aeronaves e Manut" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="610" uniqueCount="311">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="605" uniqueCount="306">
   <si>
     <t>PARÂMETRO</t>
   </si>
@@ -512,15 +512,6 @@
     <t>Warning</t>
   </si>
   <si>
-    <t>Presença de limalhas na AGB (Caixa de Acessórios) e na RGB (Caixa de</t>
-  </si>
-  <si>
-    <t>Redução), ou funcionamento anormal do motor com detecção de limal-</t>
-  </si>
-  <si>
-    <t>has ou na AGB ou na RGB.</t>
-  </si>
-  <si>
     <t>8 </t>
   </si>
   <si>
@@ -686,15 +677,6 @@
     <t>Caution</t>
   </si>
   <si>
-    <t>Presença de limalhas na RGB com funcionamento normal do motor; ou</t>
-  </si>
-  <si>
-    <t>detecção de limalhas na AGB ou na RGB com funcionamento do motor e</t>
-  </si>
-  <si>
-    <t>aeronave em solo</t>
-  </si>
-  <si>
     <t>27 </t>
   </si>
   <si>
@@ -737,12 +719,6 @@
     <t>EMER GEAR </t>
   </si>
   <si>
-    <t>Baixa pressão no acumulador de emergência que alimenta o trem de</t>
-  </si>
-  <si>
-    <t>pouso</t>
-  </si>
-  <si>
     <t>32 </t>
   </si>
   <si>
@@ -954,13 +930,22 @@
   </si>
   <si>
     <t>Bomba do tanque da fuselagem inoperante e baixo nível de combustível nos tanques das asas</t>
+  </si>
+  <si>
+    <t>Presença de limalhas na RGB com funcionamento normal do motor; ou detecção de limalhas na AGB ou na RGB com funcionamento do motor e aeronave em solo</t>
+  </si>
+  <si>
+    <t>Baixa pressão no acumulador de emergência que alimenta o trem de pouso</t>
+  </si>
+  <si>
+    <t>Presença de limalhas na AGB (Caixa de Acessórios) e na RGB (Caixa de Redução), ou funcionamento anormal do motor com detecção de limalhas ou na AGB ou na RGB.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -979,6 +964,14 @@
       <color rgb="FF000000"/>
       <name val="Helvetica"/>
       <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -1001,11 +994,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1225,12 +1224,14 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:G55"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr defaultColWidth="12.7109375" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="15.83203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="31.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="43.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1253,7 +1254,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>7</v>
       </c>
@@ -1276,7 +1277,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="3" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>12</v>
       </c>
@@ -1299,7 +1300,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="4" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>16</v>
       </c>
@@ -1322,7 +1323,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="5" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>20</v>
       </c>
@@ -1345,7 +1346,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="6" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>24</v>
       </c>
@@ -1368,7 +1369,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="7" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>29</v>
       </c>
@@ -1391,7 +1392,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="8" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>35</v>
       </c>
@@ -1414,7 +1415,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="9" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>37</v>
       </c>
@@ -1437,7 +1438,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="10" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>39</v>
       </c>
@@ -1460,7 +1461,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="11" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>41</v>
       </c>
@@ -1483,7 +1484,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="12" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
         <v>43</v>
       </c>
@@ -1506,7 +1507,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="13" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
         <v>45</v>
       </c>
@@ -1529,7 +1530,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="14" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
         <v>47</v>
       </c>
@@ -1552,7 +1553,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="15" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
         <v>49</v>
       </c>
@@ -1575,7 +1576,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="16" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="16" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
         <v>51</v>
       </c>
@@ -1598,7 +1599,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="17" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="17" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
         <v>53</v>
       </c>
@@ -1621,7 +1622,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="18" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="18" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
         <v>55</v>
       </c>
@@ -1644,7 +1645,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="19" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
         <v>57</v>
       </c>
@@ -1667,7 +1668,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="20" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="20" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
         <v>59</v>
       </c>
@@ -1690,7 +1691,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="21" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="21" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
         <v>61</v>
       </c>
@@ -1713,7 +1714,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="22" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="22" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
         <v>63</v>
       </c>
@@ -1736,7 +1737,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="23" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="23" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
         <v>65</v>
       </c>
@@ -1759,7 +1760,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="24" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="24" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
         <v>69</v>
       </c>
@@ -1782,7 +1783,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="25" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="25" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
         <v>72</v>
       </c>
@@ -1805,7 +1806,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="26" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="26" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
         <v>74</v>
       </c>
@@ -1828,7 +1829,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="27" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="27" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="1" t="s">
         <v>76</v>
       </c>
@@ -1851,7 +1852,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="28" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="28" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
         <v>78</v>
       </c>
@@ -1874,7 +1875,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="29" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="29" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="1" t="s">
         <v>80</v>
       </c>
@@ -1897,7 +1898,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="30" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="30" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="1" t="s">
         <v>82</v>
       </c>
@@ -1920,7 +1921,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="31" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="31" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="1" t="s">
         <v>84</v>
       </c>
@@ -1943,7 +1944,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="32" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="32" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="1" t="s">
         <v>86</v>
       </c>
@@ -1966,7 +1967,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="33" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="33" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="1" t="s">
         <v>88</v>
       </c>
@@ -1989,7 +1990,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="34" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="34" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="1" t="s">
         <v>90</v>
       </c>
@@ -2012,7 +2013,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="35" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="35" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="1" t="s">
         <v>92</v>
       </c>
@@ -2035,7 +2036,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="36" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="36" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="1" t="s">
         <v>94</v>
       </c>
@@ -2058,7 +2059,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="37" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="37" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="1" t="s">
         <v>96</v>
       </c>
@@ -2081,7 +2082,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="38" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="38" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="1" t="s">
         <v>98</v>
       </c>
@@ -2104,7 +2105,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="39" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="39" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="1" t="s">
         <v>100</v>
       </c>
@@ -2127,7 +2128,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="40" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="40" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="1" t="s">
         <v>104</v>
       </c>
@@ -2150,7 +2151,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="41" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="41" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="1" t="s">
         <v>107</v>
       </c>
@@ -2173,7 +2174,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="42" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="42" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="1" t="s">
         <v>109</v>
       </c>
@@ -2196,7 +2197,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="43" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="43" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="1" t="s">
         <v>111</v>
       </c>
@@ -2219,7 +2220,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="44" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="44" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="1" t="s">
         <v>113</v>
       </c>
@@ -2242,7 +2243,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="45" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="45" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="1" t="s">
         <v>115</v>
       </c>
@@ -2265,7 +2266,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="46" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="46" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="1" t="s">
         <v>117</v>
       </c>
@@ -2288,7 +2289,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="47" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="47" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="1" t="s">
         <v>119</v>
       </c>
@@ -2311,7 +2312,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="48" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="48" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="1" t="s">
         <v>121</v>
       </c>
@@ -2334,7 +2335,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="49" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="49" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="1" t="s">
         <v>123</v>
       </c>
@@ -2357,7 +2358,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="50" spans="1:7" ht="13" x14ac:dyDescent="0.15">
+    <row r="50" spans="1:7" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A50" s="1" t="s">
         <v>125</v>
       </c>
@@ -2380,7 +2381,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="51" spans="1:7" ht="13" x14ac:dyDescent="0.15">
+    <row r="51" spans="1:7" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A51" s="1" t="s">
         <v>127</v>
       </c>
@@ -2403,7 +2404,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="52" spans="1:7" ht="13" x14ac:dyDescent="0.15">
+    <row r="52" spans="1:7" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A52" s="1" t="s">
         <v>129</v>
       </c>
@@ -2426,7 +2427,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="53" spans="1:7" ht="13" x14ac:dyDescent="0.15">
+    <row r="53" spans="1:7" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A53" s="1" t="s">
         <v>131</v>
       </c>
@@ -2449,7 +2450,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="54" spans="1:7" ht="13" x14ac:dyDescent="0.15">
+    <row r="54" spans="1:7" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A54" s="1" t="s">
         <v>133</v>
       </c>
@@ -2472,7 +2473,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="55" spans="1:7" ht="13" x14ac:dyDescent="0.15">
+    <row r="55" spans="1:7" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A55" s="1" t="s">
         <v>135</v>
       </c>
@@ -2502,28 +2503,30 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6D052209-8164-FC4E-AB5F-A44E96FCE77A}">
-  <dimension ref="A1:D60"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
+  <dimension ref="A1:H55"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="27.33203125" customWidth="1"/>
-    <col min="4" max="4" width="83.33203125" customWidth="1"/>
+    <col min="1" max="1" width="16.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="83.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:8" s="5" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="A1" s="4" t="s">
         <v>137</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="4" t="s">
         <v>138</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="4" t="s">
         <v>139</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="4" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:8" ht="15" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>141</v>
       </c>
@@ -2537,7 +2540,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:8" ht="15" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>145</v>
       </c>
@@ -2551,7 +2554,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:8" ht="15" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>148</v>
       </c>
@@ -2565,7 +2568,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:8" ht="15" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>151</v>
       </c>
@@ -2579,7 +2582,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:8" ht="15" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>154</v>
       </c>
@@ -2593,7 +2596,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:8" ht="15" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>157</v>
       </c>
@@ -2607,719 +2610,681 @@
         <v>159</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A8" s="3" t="s">
+    <row r="8" spans="1:8" ht="15" x14ac:dyDescent="0.2">
+      <c r="A8" s="2" t="s">
         <v>160</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="2" t="s">
         <v>162</v>
       </c>
       <c r="D8" s="2" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="15" x14ac:dyDescent="0.2">
+      <c r="A9" s="2" t="s">
         <v>163</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A9" s="3"/>
-      <c r="B9" s="3"/>
-      <c r="C9" s="3"/>
+      <c r="B9" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>143</v>
+      </c>
       <c r="D9" s="2" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A10" s="3"/>
-      <c r="B10" s="3"/>
-      <c r="C10" s="3"/>
+        <v>165</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="15" x14ac:dyDescent="0.2">
+      <c r="A10" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>143</v>
+      </c>
       <c r="D10" s="2" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="15" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>143</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="15" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>143</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="15" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>143</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A14" s="3" t="s">
-        <v>175</v>
-      </c>
-      <c r="B14" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="H13" s="3"/>
+    </row>
+    <row r="14" spans="1:8" ht="15" x14ac:dyDescent="0.2">
+      <c r="A14" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="C14" s="2" t="s">
         <v>143</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>310</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" ht="15" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>143</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" ht="15" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>143</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="C17" s="2" t="s">
         <v>143</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="C18" s="2" t="s">
         <v>143</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>143</v>
+        <v>194</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>143</v>
+        <v>194</v>
       </c>
       <c r="D20" s="2" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" ht="15" x14ac:dyDescent="0.2">
+      <c r="A21" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="C21" s="2" t="s">
         <v>194</v>
       </c>
-    </row>
-    <row r="21" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A21" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>196</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>197</v>
-      </c>
       <c r="D21" s="2" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A23" s="2" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>212</v>
+        <v>152</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A27" s="2" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>215</v>
+        <v>161</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>197</v>
+        <v>217</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A28" s="2" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>152</v>
+        <v>219</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>218</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A29" s="3" t="s">
-        <v>219</v>
-      </c>
-      <c r="B29" s="3" t="s">
-        <v>161</v>
-      </c>
-      <c r="C29" s="3" t="s">
         <v>220</v>
       </c>
+    </row>
+    <row r="29" spans="1:4" ht="15" x14ac:dyDescent="0.2">
+      <c r="A29" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>194</v>
+      </c>
       <c r="D29" s="2" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A30" s="3"/>
-      <c r="B30" s="3"/>
-      <c r="C30" s="3"/>
+        <v>223</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" ht="15" x14ac:dyDescent="0.2">
+      <c r="A30" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>194</v>
+      </c>
       <c r="D30" s="2" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A31" s="3"/>
-      <c r="B31" s="3"/>
-      <c r="C31" s="3"/>
+        <v>226</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" ht="15" x14ac:dyDescent="0.2">
+      <c r="A31" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>194</v>
+      </c>
       <c r="D31" s="2" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A32" s="2" t="s">
-        <v>224</v>
+        <v>230</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>225</v>
+        <v>231</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>226</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A33" s="2" t="s">
-        <v>227</v>
+        <v>232</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>228</v>
+        <v>233</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A34" s="2" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>231</v>
+        <v>236</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A35" s="2" t="s">
-        <v>233</v>
+        <v>238</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>235</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A36" s="3" t="s">
-        <v>236</v>
-      </c>
-      <c r="B36" s="3" t="s">
-        <v>237</v>
-      </c>
-      <c r="C36" s="3" t="s">
-        <v>197</v>
+        <v>240</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" ht="15" x14ac:dyDescent="0.2">
+      <c r="A36" s="2" t="s">
+        <v>241</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>194</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A37" s="3"/>
-      <c r="B37" s="3"/>
-      <c r="C37" s="3"/>
+        <v>243</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" ht="15" x14ac:dyDescent="0.2">
+      <c r="A37" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>194</v>
+      </c>
       <c r="D37" s="2" t="s">
-        <v>239</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A38" s="2" t="s">
-        <v>240</v>
+        <v>247</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>241</v>
+        <v>248</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A39" s="2" t="s">
-        <v>243</v>
+        <v>250</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>244</v>
+        <v>251</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A40" s="2" t="s">
-        <v>246</v>
+        <v>253</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>247</v>
+        <v>254</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A41" s="2" t="s">
-        <v>249</v>
+        <v>256</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>250</v>
+        <v>257</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A42" s="2" t="s">
-        <v>252</v>
+        <v>259</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>253</v>
+        <v>260</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A43" s="2" t="s">
-        <v>255</v>
+        <v>262</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>256</v>
+        <v>263</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>257</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A44" s="2" t="s">
-        <v>258</v>
+        <v>264</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>259</v>
+        <v>265</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>260</v>
-      </c>
-    </row>
-    <row r="45" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A45" s="2" t="s">
-        <v>261</v>
+        <v>267</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>262</v>
+        <v>268</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A46" s="2" t="s">
-        <v>264</v>
+        <v>270</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A47" s="2" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="48" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A48" s="3" t="s">
-        <v>270</v>
-      </c>
-      <c r="B48" s="3" t="s">
-        <v>271</v>
-      </c>
-      <c r="C48" s="3" t="s">
-        <v>197</v>
+        <v>275</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" ht="15" x14ac:dyDescent="0.2">
+      <c r="A48" s="2" t="s">
+        <v>276</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="C48" s="2" t="s">
+        <v>194</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>309</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A49" s="3" t="s">
-        <v>272</v>
-      </c>
-      <c r="B49" s="3" t="s">
-        <v>273</v>
-      </c>
-      <c r="C49" s="3" t="s">
-        <v>197</v>
+        <v>278</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" ht="15" x14ac:dyDescent="0.2">
+      <c r="A49" s="2" t="s">
+        <v>279</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="C49" s="2" t="s">
+        <v>194</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>274</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A50" s="2" t="s">
-        <v>275</v>
+        <v>282</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>276</v>
+        <v>283</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>197</v>
+        <v>284</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="51" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A51" s="2" t="s">
-        <v>278</v>
+        <v>286</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>279</v>
+        <v>287</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>197</v>
+        <v>284</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>280</v>
-      </c>
-    </row>
-    <row r="52" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A52" s="2" t="s">
-        <v>281</v>
+        <v>289</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>282</v>
+        <v>290</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>197</v>
+        <v>284</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>283</v>
-      </c>
-    </row>
-    <row r="53" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A53" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="B53" s="2" t="s">
+        <v>293</v>
+      </c>
+      <c r="C53" s="2" t="s">
         <v>284</v>
       </c>
-      <c r="B53" s="2" t="s">
-        <v>285</v>
-      </c>
-      <c r="C53" s="2" t="s">
-        <v>197</v>
-      </c>
       <c r="D53" s="2" t="s">
-        <v>286</v>
-      </c>
-    </row>
-    <row r="54" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A54" s="2" t="s">
-        <v>287</v>
+        <v>295</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>288</v>
+        <v>296</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>197</v>
+        <v>284</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="55" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" ht="15" x14ac:dyDescent="0.2">
       <c r="A55" s="2" t="s">
-        <v>290</v>
+        <v>298</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>291</v>
+        <v>299</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>292</v>
+        <v>284</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>293</v>
-      </c>
-    </row>
-    <row r="56" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A56" s="2" t="s">
-        <v>294</v>
-      </c>
-      <c r="B56" s="2" t="s">
-        <v>295</v>
-      </c>
-      <c r="C56" s="2" t="s">
-        <v>292</v>
-      </c>
-      <c r="D56" s="2" t="s">
-        <v>296</v>
-      </c>
-    </row>
-    <row r="57" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A57" s="2" t="s">
-        <v>297</v>
-      </c>
-      <c r="B57" s="2" t="s">
-        <v>298</v>
-      </c>
-      <c r="C57" s="2" t="s">
-        <v>292</v>
-      </c>
-      <c r="D57" s="2" t="s">
-        <v>299</v>
-      </c>
-    </row>
-    <row r="58" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A58" s="2" t="s">
         <v>300</v>
-      </c>
-      <c r="B58" s="2" t="s">
-        <v>301</v>
-      </c>
-      <c r="C58" s="2" t="s">
-        <v>292</v>
-      </c>
-      <c r="D58" s="2" t="s">
-        <v>302</v>
-      </c>
-    </row>
-    <row r="59" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A59" s="2" t="s">
-        <v>303</v>
-      </c>
-      <c r="B59" s="2" t="s">
-        <v>304</v>
-      </c>
-      <c r="C59" s="2" t="s">
-        <v>292</v>
-      </c>
-      <c r="D59" s="2" t="s">
-        <v>305</v>
-      </c>
-    </row>
-    <row r="60" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A60" s="2" t="s">
-        <v>306</v>
-      </c>
-      <c r="B60" s="2" t="s">
-        <v>307</v>
-      </c>
-      <c r="C60" s="2" t="s">
-        <v>292</v>
-      </c>
-      <c r="D60" s="2" t="s">
-        <v>308</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(app): menu duplication (B-01) and y_col validation (B-02); feat: optimize I/O and phase detection (S-01 to S-06)
</commit_message>
<xml_diff>
--- a/docs/Parâmetros de Aeronaves e Manutenção.xlsx
+++ b/docs/Parâmetros de Aeronaves e Manutenção.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\brgar\Projetos\VADER\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3520DD0E-5AF1-430C-91DC-B4E99960E03D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{416781AB-59F7-47D3-84D3-2BBD78E44CD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="16800" yWindow="0" windowWidth="24450" windowHeight="15345" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="605" uniqueCount="306">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="550" uniqueCount="251">
   <si>
     <t>PARÂMETRO</t>
   </si>
@@ -434,9 +434,6 @@
     <t>Falha do solenoide de corte.</t>
   </si>
   <si>
-    <t>REFERÊNCIA </t>
-  </si>
-  <si>
     <t>MENSAGEM </t>
   </si>
   <si>
@@ -446,9 +443,6 @@
     <t>EXPLICAÇÃO</t>
   </si>
   <si>
-    <t>1 </t>
-  </si>
-  <si>
     <t>AP </t>
   </si>
   <si>
@@ -458,150 +452,99 @@
     <t>Falha no piloto automático</t>
   </si>
   <si>
-    <t>2 </t>
-  </si>
-  <si>
     <t>BAT TEMP </t>
   </si>
   <si>
     <t>Temperatura elevada da bateria</t>
   </si>
   <si>
-    <t>3 </t>
-  </si>
-  <si>
     <t>BLD LEAK </t>
   </si>
   <si>
     <t>Vazamento no sistema de sangria de ar do motor</t>
   </si>
   <si>
-    <t>4 </t>
-  </si>
-  <si>
     <t>CAB ALT </t>
   </si>
   <si>
     <t>Altitude elevada da cabine (maior do que 25000ft)</t>
   </si>
   <si>
-    <t>5 </t>
-  </si>
-  <si>
     <t>CAB PRES </t>
   </si>
   <si>
     <t>Sobrepressão na cabine</t>
   </si>
   <si>
-    <t>6 </t>
-  </si>
-  <si>
     <t>CANOPY </t>
   </si>
   <si>
     <t>Capota aberta</t>
   </si>
   <si>
-    <t>7 </t>
-  </si>
-  <si>
     <t>CHIP DET </t>
   </si>
   <si>
     <t>Warning</t>
   </si>
   <si>
-    <t>8 </t>
-  </si>
-  <si>
     <t>ENG MAN </t>
   </si>
   <si>
     <t>Falha na PMU</t>
   </si>
   <si>
-    <t>9 </t>
-  </si>
-  <si>
     <t>ENG LMTS </t>
   </si>
   <si>
     <t>Limites do motor alcançados</t>
   </si>
   <si>
-    <t>10 </t>
-  </si>
-  <si>
     <t>FIRE </t>
   </si>
   <si>
     <t>Fogo detectado no motor</t>
   </si>
   <si>
-    <t>11 </t>
-  </si>
-  <si>
     <t>FUEL FUS </t>
   </si>
   <si>
-    <t>12 </t>
-  </si>
-  <si>
     <t>FUEL LVL </t>
   </si>
   <si>
     <t>Baixo nível de combustível</t>
   </si>
   <si>
-    <t>13 </t>
-  </si>
-  <si>
     <t>FWD OXY </t>
   </si>
   <si>
     <t>Anormalidade no regulador de oxigênio</t>
   </si>
   <si>
-    <t>14 </t>
-  </si>
-  <si>
     <t>LDG GEAR </t>
   </si>
   <si>
     <t>Trem de pouso recolhido, quando deveria estar estendido</t>
   </si>
   <si>
-    <t>15 </t>
-  </si>
-  <si>
     <t>OIL PRES </t>
   </si>
   <si>
     <t>Baixa/Alta pressão do óleo</t>
   </si>
   <si>
-    <t>16 </t>
-  </si>
-  <si>
     <t>OIL TEMP </t>
   </si>
   <si>
     <t>Baixa/Alta temperatura do óleo</t>
   </si>
   <si>
-    <t>17 </t>
-  </si>
-  <si>
     <t>OXYGEN </t>
   </si>
   <si>
     <t>Baixa pressão de saída de oxigênio do concentrador</t>
   </si>
   <si>
-    <t>18 </t>
-  </si>
-  <si>
     <t>AIR COND </t>
   </si>
   <si>
@@ -611,267 +554,174 @@
     <t>Falha no condicionamento de ar</t>
   </si>
   <si>
-    <t>19 </t>
-  </si>
-  <si>
     <t>AP MIST </t>
   </si>
   <si>
     <t>Falha na compensação do piloto automático</t>
   </si>
   <si>
-    <t>20 </t>
-  </si>
-  <si>
     <t>AVIONICS </t>
   </si>
   <si>
     <t>Mau funcionamento de algum equipamento aviônico</t>
   </si>
   <si>
-    <t>21 </t>
-  </si>
-  <si>
     <t>BATTERY </t>
   </si>
   <si>
     <t>Bateria principal sendo descarregada</t>
   </si>
   <si>
-    <t>22 </t>
-  </si>
-  <si>
     <t>BINGO </t>
   </si>
   <si>
     <t>Combustível remanescente não é suficiente para retorno à base</t>
   </si>
   <si>
-    <t>23 </t>
-  </si>
-  <si>
     <t>BKUP BAT </t>
   </si>
   <si>
     <t>Falha no sistema da bateria de reserva</t>
   </si>
   <si>
-    <t>24 </t>
-  </si>
-  <si>
     <t>BLD OVHT </t>
   </si>
   <si>
     <t>Sobreaquecimento no sistema de sangria de ar do motor</t>
   </si>
   <si>
-    <t>25 </t>
-  </si>
-  <si>
     <t>Descompressão da cabine (limite de 16000ft excedido)</t>
   </si>
   <si>
-    <t>26 </t>
-  </si>
-  <si>
     <t>Caution</t>
   </si>
   <si>
-    <t>27 </t>
-  </si>
-  <si>
     <t>ELEC XFR </t>
   </si>
   <si>
     <t>Falha na transferência para a condição de emergência elétrica</t>
   </si>
   <si>
-    <t>28 </t>
-  </si>
-  <si>
     <t>ELEK OVH </t>
   </si>
   <si>
     <t>Sobreaquecimento no compartimento eletrônico</t>
   </si>
   <si>
-    <t>29 </t>
-  </si>
-  <si>
     <t>EMER BRK </t>
   </si>
   <si>
     <t>Baixa pressão no sistema do freio de emergência</t>
   </si>
   <si>
-    <t>30 </t>
-  </si>
-  <si>
     <t>EMER BUS </t>
   </si>
   <si>
     <t>Barra de emergência desenergizada</t>
   </si>
   <si>
-    <t>31 </t>
-  </si>
-  <si>
     <t>EMER GEAR </t>
   </si>
   <si>
-    <t>32 </t>
-  </si>
-  <si>
     <t>FUEL IMB </t>
   </si>
   <si>
     <t>Combustível desbalanceado</t>
   </si>
   <si>
-    <t>33 </t>
-  </si>
-  <si>
     <t>FUEL XFER </t>
   </si>
   <si>
     <t>Falha na transferência de combustível</t>
   </si>
   <si>
-    <t>34 </t>
-  </si>
-  <si>
     <t>FUEL FILT </t>
   </si>
   <si>
     <t>Passagem secundária iminente no filtro de combustível</t>
   </si>
   <si>
-    <t>35 </t>
-  </si>
-  <si>
     <t>FUEL PRES </t>
   </si>
   <si>
     <t>Baixa pressão do combustível</t>
   </si>
   <si>
-    <t>36 </t>
-  </si>
-  <si>
     <t>FUS LVL </t>
   </si>
   <si>
     <t>Baixo nível de combustível no tanque da fuselagem</t>
   </si>
   <si>
-    <t>37 </t>
-  </si>
-  <si>
     <t>FWD PIN </t>
   </si>
   <si>
     <t>Pino de segurança instalado no assento</t>
   </si>
   <si>
-    <t>38 </t>
-  </si>
-  <si>
     <t>GB OVLD </t>
   </si>
   <si>
     <t>Sobrecarga na caixa de engrenagens</t>
   </si>
   <si>
-    <t>39 </t>
-  </si>
-  <si>
     <t>GEN </t>
   </si>
   <si>
     <t>Gerador fora da barra</t>
   </si>
   <si>
-    <t>40 </t>
-  </si>
-  <si>
     <t>HYD PRES </t>
   </si>
   <si>
     <t>Baixa/Alta pressão hidráulica</t>
   </si>
   <si>
-    <t>41 </t>
-  </si>
-  <si>
     <t>LWING LVL </t>
   </si>
   <si>
     <t>Baixo nível de combustível no tanque da asa esquerda</t>
   </si>
   <si>
-    <t>42 </t>
-  </si>
-  <si>
     <t>MAN RUD T </t>
   </si>
   <si>
-    <t>43 </t>
-  </si>
-  <si>
     <t>PITO TAT </t>
   </si>
   <si>
     <t>Falha no sistema de aquecimento primário do Pitot/TAT</t>
   </si>
   <si>
-    <t>44 </t>
-  </si>
-  <si>
     <t>PROP DEIC </t>
   </si>
   <si>
     <t>O degelador da hélice deve ser acionado</t>
   </si>
   <si>
-    <t>45 </t>
-  </si>
-  <si>
     <t>RWING LVL </t>
   </si>
   <si>
     <t>Baixo nível de combustível no tanque da asa direita</t>
   </si>
   <si>
-    <t>46 </t>
-  </si>
-  <si>
     <t>S PITOT </t>
   </si>
   <si>
     <t>Falha no sistema de aquecimento secundário do Pitot</t>
   </si>
   <si>
-    <t>47 </t>
-  </si>
-  <si>
     <t>STARTER </t>
   </si>
   <si>
     <t>Falha no(s) contactor(es) de partida do motor</t>
   </si>
   <si>
-    <t>48 </t>
-  </si>
-  <si>
     <t>STORM </t>
   </si>
   <si>
     <t>Aparecimento de nuvem carregada com eletricidade</t>
   </si>
   <si>
-    <t>49 </t>
-  </si>
-  <si>
     <t>INERT SEP </t>
   </si>
   <si>
@@ -881,43 +731,28 @@
     <t>Separação inercial ativada</t>
   </si>
   <si>
-    <t>50 </t>
-  </si>
-  <si>
     <t>INTC ON </t>
   </si>
   <si>
     <t>Interconexão com outra aeronave em execução</t>
   </si>
   <si>
-    <t>51 </t>
-  </si>
-  <si>
     <t>OXYBIT </t>
   </si>
   <si>
     <t>Autoteste do OBOGS (Sistema de Geração de Oxigênio) em execução</t>
   </si>
   <si>
-    <t>52 </t>
-  </si>
-  <si>
     <t>XFER OVRD </t>
   </si>
   <si>
     <t>Transferência automática de combustível sobrepujada</t>
   </si>
   <si>
-    <t>53 </t>
-  </si>
-  <si>
     <t>WING CLOS </t>
   </si>
   <si>
     <t>Válvula de isolamento dos tanques de asa totalmente fechada</t>
-  </si>
-  <si>
-    <t>54 </t>
   </si>
   <si>
     <t>WS DEICE </t>
@@ -2503,16 +2338,15 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6D052209-8164-FC4E-AB5F-A44E96FCE77A}">
-  <dimension ref="A1:H55"/>
+  <dimension ref="A1:G55"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="16.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="83.28515625" customWidth="1"/>
+    <col min="1" max="1" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="177.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="5" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" s="5" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
         <v>137</v>
       </c>
@@ -2522,765 +2356,600 @@
       <c r="C1" s="4" t="s">
         <v>139</v>
       </c>
-      <c r="D1" s="4" t="s">
+    </row>
+    <row r="2" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="A2" s="2" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" ht="15" x14ac:dyDescent="0.2">
-      <c r="A2" s="2" t="s">
+      <c r="B2" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="C2" s="2" t="s">
+    </row>
+    <row r="3" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="A3" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="B3" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="15" x14ac:dyDescent="0.2">
-      <c r="A3" s="2" t="s">
+    <row r="4" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="A4" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B4" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="D3" s="2" t="s">
+    </row>
+    <row r="5" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="A5" s="2" t="s">
         <v>147</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" ht="15" x14ac:dyDescent="0.2">
-      <c r="A4" s="2" t="s">
+      <c r="B5" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="B4" s="2" t="s">
+    </row>
+    <row r="6" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="A6" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="C4" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="D4" s="2" t="s">
+      <c r="B6" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="15" x14ac:dyDescent="0.2">
-      <c r="A5" s="2" t="s">
+    <row r="7" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="A7" s="2" t="s">
         <v>151</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B7" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="C5" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="D5" s="2" t="s">
+    </row>
+    <row r="8" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="A8" s="2" t="s">
         <v>153</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" ht="15" x14ac:dyDescent="0.2">
-      <c r="A6" s="2" t="s">
+      <c r="B8" s="2" t="s">
         <v>154</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="C8" s="2" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="A9" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="D6" s="2" t="s">
+      <c r="B9" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="15" x14ac:dyDescent="0.2">
-      <c r="A7" s="2" t="s">
+    <row r="10" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="A10" s="2" t="s">
         <v>157</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B10" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>158</v>
       </c>
-      <c r="C7" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="D7" s="2" t="s">
+    </row>
+    <row r="11" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="A11" s="2" t="s">
         <v>159</v>
       </c>
-    </row>
-    <row r="8" spans="1:8" ht="15" x14ac:dyDescent="0.2">
-      <c r="A8" s="2" t="s">
+      <c r="B11" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="C11" s="2" t="s">
         <v>160</v>
       </c>
-      <c r="B8" s="2" t="s">
+    </row>
+    <row r="12" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="A12" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="B12" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="A13" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="D8" s="2" t="s">
-        <v>305</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" ht="15" x14ac:dyDescent="0.2">
-      <c r="A9" s="2" t="s">
+      <c r="B13" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="C13" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="G13" s="3"/>
+    </row>
+    <row r="14" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="A14" s="2" t="s">
         <v>164</v>
       </c>
-      <c r="C9" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="D9" s="2" t="s">
+      <c r="B14" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="C14" s="2" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="15" x14ac:dyDescent="0.2">
-      <c r="A10" s="2" t="s">
+    <row r="15" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="A15" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B15" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="C15" s="2" t="s">
         <v>167</v>
       </c>
-      <c r="C10" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="D10" s="2" t="s">
+    </row>
+    <row r="16" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="A16" s="2" t="s">
         <v>168</v>
       </c>
-    </row>
-    <row r="11" spans="1:8" ht="15" x14ac:dyDescent="0.2">
-      <c r="A11" s="2" t="s">
+      <c r="B16" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="C16" s="2" t="s">
         <v>169</v>
       </c>
-      <c r="B11" s="2" t="s">
+    </row>
+    <row r="17" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A17" s="2" t="s">
         <v>170</v>
       </c>
-      <c r="C11" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="D11" s="2" t="s">
+      <c r="B17" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="C17" s="2" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="15" x14ac:dyDescent="0.2">
-      <c r="A12" s="2" t="s">
+    <row r="18" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A18" s="2" t="s">
         <v>172</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B18" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="C18" s="2" t="s">
         <v>173</v>
       </c>
-      <c r="C12" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>302</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" ht="15" x14ac:dyDescent="0.2">
-      <c r="A13" s="2" t="s">
+    </row>
+    <row r="19" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A19" s="2" t="s">
         <v>174</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B19" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="C13" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="D13" s="2" t="s">
+      <c r="C19" s="2" t="s">
         <v>176</v>
       </c>
-      <c r="H13" s="3"/>
-    </row>
-    <row r="14" spans="1:8" ht="15" x14ac:dyDescent="0.2">
-      <c r="A14" s="2" t="s">
+    </row>
+    <row r="20" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A20" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B20" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="C20" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="C14" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="D14" s="2" t="s">
+    </row>
+    <row r="21" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A21" s="2" t="s">
         <v>179</v>
       </c>
-    </row>
-    <row r="15" spans="1:8" ht="15" x14ac:dyDescent="0.2">
-      <c r="A15" s="2" t="s">
+      <c r="B21" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="C21" s="2" t="s">
         <v>180</v>
       </c>
-      <c r="B15" s="2" t="s">
+    </row>
+    <row r="22" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A22" s="2" t="s">
         <v>181</v>
       </c>
-      <c r="C15" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="D15" s="2" t="s">
+      <c r="B22" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="C22" s="2" t="s">
         <v>182</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="15" x14ac:dyDescent="0.2">
-      <c r="A16" s="2" t="s">
+    <row r="23" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A23" s="2" t="s">
         <v>183</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B23" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="C23" s="2" t="s">
         <v>184</v>
       </c>
-      <c r="C16" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="D16" s="2" t="s">
+    </row>
+    <row r="24" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A24" s="2" t="s">
         <v>185</v>
       </c>
-    </row>
-    <row r="17" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A17" s="2" t="s">
+      <c r="B24" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="C24" s="2" t="s">
         <v>186</v>
       </c>
-      <c r="B17" s="2" t="s">
+    </row>
+    <row r="25" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A25" s="2" t="s">
         <v>187</v>
       </c>
-      <c r="C17" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="D17" s="2" t="s">
+      <c r="B25" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="C25" s="2" t="s">
         <v>188</v>
       </c>
     </row>
-    <row r="18" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A18" s="2" t="s">
+    <row r="26" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A26" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="C26" s="2" t="s">
         <v>189</v>
       </c>
-      <c r="B18" s="2" t="s">
+    </row>
+    <row r="27" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A27" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="B27" s="2" t="s">
         <v>190</v>
       </c>
-      <c r="C18" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="D18" s="2" t="s">
+      <c r="C27" s="2" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A28" s="2" t="s">
         <v>191</v>
       </c>
-    </row>
-    <row r="19" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A19" s="2" t="s">
+      <c r="B28" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="C28" s="2" t="s">
         <v>192</v>
       </c>
-      <c r="B19" s="2" t="s">
+    </row>
+    <row r="29" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A29" s="2" t="s">
         <v>193</v>
       </c>
-      <c r="C19" s="2" t="s">
-        <v>194</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A20" s="2" t="s">
-        <v>196</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>194</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A21" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>200</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>194</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A22" s="2" t="s">
-        <v>202</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>203</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>194</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A23" s="2" t="s">
-        <v>205</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>206</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>194</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A24" s="2" t="s">
-        <v>208</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>209</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>194</v>
-      </c>
-      <c r="D24" s="2" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A25" s="2" t="s">
-        <v>211</v>
-      </c>
-      <c r="B25" s="2" t="s">
-        <v>212</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>194</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A26" s="2" t="s">
-        <v>214</v>
-      </c>
-      <c r="B26" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="C26" s="2" t="s">
-        <v>194</v>
-      </c>
-      <c r="D26" s="2" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A27" s="2" t="s">
-        <v>216</v>
-      </c>
-      <c r="B27" s="2" t="s">
-        <v>161</v>
-      </c>
-      <c r="C27" s="2" t="s">
-        <v>217</v>
-      </c>
-      <c r="D27" s="2" t="s">
-        <v>303</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A28" s="2" t="s">
-        <v>218</v>
-      </c>
-      <c r="B28" s="2" t="s">
-        <v>219</v>
-      </c>
-      <c r="C28" s="2" t="s">
-        <v>194</v>
-      </c>
-      <c r="D28" s="2" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A29" s="2" t="s">
-        <v>221</v>
-      </c>
       <c r="B29" s="2" t="s">
-        <v>222</v>
+        <v>175</v>
       </c>
       <c r="C29" s="2" t="s">
         <v>194</v>
       </c>
-      <c r="D29" s="2" t="s">
+    </row>
+    <row r="30" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A30" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A31" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A32" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A33" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A34" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A35" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A36" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A37" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A38" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A39" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A40" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A41" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A42" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A43" s="2" t="s">
+        <v>220</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A44" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A45" s="2" t="s">
         <v>223</v>
       </c>
-    </row>
-    <row r="30" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A30" s="2" t="s">
+      <c r="B45" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="C45" s="2" t="s">
         <v>224</v>
       </c>
-      <c r="B30" s="2" t="s">
+    </row>
+    <row r="46" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A46" s="2" t="s">
         <v>225</v>
       </c>
-      <c r="C30" s="2" t="s">
-        <v>194</v>
-      </c>
-      <c r="D30" s="2" t="s">
+      <c r="B46" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="C46" s="2" t="s">
         <v>226</v>
       </c>
     </row>
-    <row r="31" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A31" s="2" t="s">
+    <row r="47" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A47" s="2" t="s">
         <v>227</v>
       </c>
-      <c r="B31" s="2" t="s">
+      <c r="B47" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="C47" s="2" t="s">
         <v>228</v>
       </c>
-      <c r="C31" s="2" t="s">
-        <v>194</v>
-      </c>
-      <c r="D31" s="2" t="s">
+    </row>
+    <row r="48" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A48" s="2" t="s">
         <v>229</v>
       </c>
-    </row>
-    <row r="32" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A32" s="2" t="s">
+      <c r="B48" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="C48" s="2" t="s">
         <v>230</v>
       </c>
-      <c r="B32" s="2" t="s">
+    </row>
+    <row r="49" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A49" s="2" t="s">
         <v>231</v>
       </c>
-      <c r="C32" s="2" t="s">
-        <v>194</v>
-      </c>
-      <c r="D32" s="2" t="s">
-        <v>304</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A33" s="2" t="s">
+      <c r="B49" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="C49" s="2" t="s">
         <v>232</v>
       </c>
-      <c r="B33" s="2" t="s">
+    </row>
+    <row r="50" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A50" s="2" t="s">
         <v>233</v>
       </c>
-      <c r="C33" s="2" t="s">
-        <v>194</v>
-      </c>
-      <c r="D33" s="2" t="s">
+      <c r="B50" s="2" t="s">
         <v>234</v>
       </c>
-    </row>
-    <row r="34" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A34" s="2" t="s">
+      <c r="C50" s="2" t="s">
         <v>235</v>
       </c>
-      <c r="B34" s="2" t="s">
+    </row>
+    <row r="51" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A51" s="2" t="s">
         <v>236</v>
       </c>
-      <c r="C34" s="2" t="s">
-        <v>194</v>
-      </c>
-      <c r="D34" s="2" t="s">
+      <c r="B51" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="C51" s="2" t="s">
         <v>237</v>
       </c>
     </row>
-    <row r="35" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A35" s="2" t="s">
+    <row r="52" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A52" s="2" t="s">
         <v>238</v>
       </c>
-      <c r="B35" s="2" t="s">
+      <c r="B52" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="C52" s="2" t="s">
         <v>239</v>
       </c>
-      <c r="C35" s="2" t="s">
-        <v>194</v>
-      </c>
-      <c r="D35" s="2" t="s">
+    </row>
+    <row r="53" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A53" s="2" t="s">
         <v>240</v>
       </c>
-    </row>
-    <row r="36" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A36" s="2" t="s">
+      <c r="B53" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="C53" s="2" t="s">
         <v>241</v>
       </c>
-      <c r="B36" s="2" t="s">
+    </row>
+    <row r="54" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A54" s="2" t="s">
         <v>242</v>
       </c>
-      <c r="C36" s="2" t="s">
-        <v>194</v>
-      </c>
-      <c r="D36" s="2" t="s">
+      <c r="B54" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="C54" s="2" t="s">
         <v>243</v>
       </c>
     </row>
-    <row r="37" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A37" s="2" t="s">
+    <row r="55" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+      <c r="A55" s="2" t="s">
         <v>244</v>
       </c>
-      <c r="B37" s="2" t="s">
+      <c r="B55" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="C55" s="2" t="s">
         <v>245</v>
-      </c>
-      <c r="C37" s="2" t="s">
-        <v>194</v>
-      </c>
-      <c r="D37" s="2" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A38" s="2" t="s">
-        <v>247</v>
-      </c>
-      <c r="B38" s="2" t="s">
-        <v>248</v>
-      </c>
-      <c r="C38" s="2" t="s">
-        <v>194</v>
-      </c>
-      <c r="D38" s="2" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A39" s="2" t="s">
-        <v>250</v>
-      </c>
-      <c r="B39" s="2" t="s">
-        <v>251</v>
-      </c>
-      <c r="C39" s="2" t="s">
-        <v>194</v>
-      </c>
-      <c r="D39" s="2" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A40" s="2" t="s">
-        <v>253</v>
-      </c>
-      <c r="B40" s="2" t="s">
-        <v>254</v>
-      </c>
-      <c r="C40" s="2" t="s">
-        <v>194</v>
-      </c>
-      <c r="D40" s="2" t="s">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A41" s="2" t="s">
-        <v>256</v>
-      </c>
-      <c r="B41" s="2" t="s">
-        <v>257</v>
-      </c>
-      <c r="C41" s="2" t="s">
-        <v>194</v>
-      </c>
-      <c r="D41" s="2" t="s">
-        <v>258</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A42" s="2" t="s">
-        <v>259</v>
-      </c>
-      <c r="B42" s="2" t="s">
-        <v>260</v>
-      </c>
-      <c r="C42" s="2" t="s">
-        <v>194</v>
-      </c>
-      <c r="D42" s="2" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A43" s="2" t="s">
-        <v>262</v>
-      </c>
-      <c r="B43" s="2" t="s">
-        <v>263</v>
-      </c>
-      <c r="C43" s="2" t="s">
-        <v>194</v>
-      </c>
-      <c r="D43" s="2" t="s">
-        <v>301</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A44" s="2" t="s">
-        <v>264</v>
-      </c>
-      <c r="B44" s="2" t="s">
-        <v>265</v>
-      </c>
-      <c r="C44" s="2" t="s">
-        <v>194</v>
-      </c>
-      <c r="D44" s="2" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="45" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A45" s="2" t="s">
-        <v>267</v>
-      </c>
-      <c r="B45" s="2" t="s">
-        <v>268</v>
-      </c>
-      <c r="C45" s="2" t="s">
-        <v>194</v>
-      </c>
-      <c r="D45" s="2" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A46" s="2" t="s">
-        <v>270</v>
-      </c>
-      <c r="B46" s="2" t="s">
-        <v>271</v>
-      </c>
-      <c r="C46" s="2" t="s">
-        <v>194</v>
-      </c>
-      <c r="D46" s="2" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A47" s="2" t="s">
-        <v>273</v>
-      </c>
-      <c r="B47" s="2" t="s">
-        <v>274</v>
-      </c>
-      <c r="C47" s="2" t="s">
-        <v>194</v>
-      </c>
-      <c r="D47" s="2" t="s">
-        <v>275</v>
-      </c>
-    </row>
-    <row r="48" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A48" s="2" t="s">
-        <v>276</v>
-      </c>
-      <c r="B48" s="2" t="s">
-        <v>277</v>
-      </c>
-      <c r="C48" s="2" t="s">
-        <v>194</v>
-      </c>
-      <c r="D48" s="2" t="s">
-        <v>278</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A49" s="2" t="s">
-        <v>279</v>
-      </c>
-      <c r="B49" s="2" t="s">
-        <v>280</v>
-      </c>
-      <c r="C49" s="2" t="s">
-        <v>194</v>
-      </c>
-      <c r="D49" s="2" t="s">
-        <v>281</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A50" s="2" t="s">
-        <v>282</v>
-      </c>
-      <c r="B50" s="2" t="s">
-        <v>283</v>
-      </c>
-      <c r="C50" s="2" t="s">
-        <v>284</v>
-      </c>
-      <c r="D50" s="2" t="s">
-        <v>285</v>
-      </c>
-    </row>
-    <row r="51" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A51" s="2" t="s">
-        <v>286</v>
-      </c>
-      <c r="B51" s="2" t="s">
-        <v>287</v>
-      </c>
-      <c r="C51" s="2" t="s">
-        <v>284</v>
-      </c>
-      <c r="D51" s="2" t="s">
-        <v>288</v>
-      </c>
-    </row>
-    <row r="52" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A52" s="2" t="s">
-        <v>289</v>
-      </c>
-      <c r="B52" s="2" t="s">
-        <v>290</v>
-      </c>
-      <c r="C52" s="2" t="s">
-        <v>284</v>
-      </c>
-      <c r="D52" s="2" t="s">
-        <v>291</v>
-      </c>
-    </row>
-    <row r="53" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A53" s="2" t="s">
-        <v>292</v>
-      </c>
-      <c r="B53" s="2" t="s">
-        <v>293</v>
-      </c>
-      <c r="C53" s="2" t="s">
-        <v>284</v>
-      </c>
-      <c r="D53" s="2" t="s">
-        <v>294</v>
-      </c>
-    </row>
-    <row r="54" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A54" s="2" t="s">
-        <v>295</v>
-      </c>
-      <c r="B54" s="2" t="s">
-        <v>296</v>
-      </c>
-      <c r="C54" s="2" t="s">
-        <v>284</v>
-      </c>
-      <c r="D54" s="2" t="s">
-        <v>297</v>
-      </c>
-    </row>
-    <row r="55" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A55" s="2" t="s">
-        <v>298</v>
-      </c>
-      <c r="B55" s="2" t="s">
-        <v>299</v>
-      </c>
-      <c r="C55" s="2" t="s">
-        <v>284</v>
-      </c>
-      <c r="D55" s="2" t="s">
-        <v>300</v>
       </c>
     </row>
   </sheetData>

</xml_diff>